<commit_message>
updqated the all excel sheet issue
</commit_message>
<xml_diff>
--- a/REPAIR_LOG_LOCAL.xlsx
+++ b/REPAIR_LOG_LOCAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\kitkart\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{733C55A6-2938-4CDF-B939-1C0E4150C573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A52645-A9A1-430D-840D-91F297D786C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
   <si>
     <t>id</t>
   </si>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t>kanika</t>
+  </si>
+  <si>
+    <t>sheik</t>
   </si>
 </sst>
 </file>
@@ -487,7 +490,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" style="4" bestFit="1" customWidth="1"/>
@@ -707,6 +710,66 @@
         <v>17</v>
       </c>
     </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="4">
+        <v>123456789</v>
+      </c>
+      <c r="E10" s="4">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="4">
+        <v>987654321</v>
+      </c>
+      <c r="E11" s="4">
+        <v>54</v>
+      </c>
+      <c r="F11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="4">
+        <v>54326789</v>
+      </c>
+      <c r="E12" s="4">
+        <v>77</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>